<commit_message>
chore: publish ekg IG 2.0.1
</commit_message>
<xml_diff>
--- a/ig/ekg/StructureDefinition-medcom-ekg-recording-bundle.xlsx
+++ b/ig/ekg/StructureDefinition-medcom-ekg-recording-bundle.xlsx
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>2.0.0</t>
+    <t>2.0.1</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-04T11:20:25+00:00</t>
+    <t>2026-10-01T09:27:07+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1315,45 +1315,45 @@
   <dimension ref="A1:AN81"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="62.49609375" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="33.44140625" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="29.421875" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="4" max="4" width="18.19140625" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="5" max="5" width="5.80859375" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="4.23828125" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="4.65625" customWidth="true" bestFit="true"/>
-    <col min="8" max="8" width="13.953125" customWidth="true" bestFit="true"/>
-    <col min="9" max="9" width="11.3671875" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="5.0" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="4" max="4" width="5.0" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="5" max="5" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="9" max="9" width="5.0" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="79.828125" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="5.0" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>
-    <col min="15" max="15" width="255.0" customWidth="true" bestFit="true"/>
+    <col min="15" max="15" width="5.0" customWidth="true" bestFit="true"/>
     <col min="16" max="16" width="20.703125" customWidth="true" bestFit="true"/>
     <col min="17" max="17" width="20.703125" customWidth="true" bestFit="true"/>
     <col min="18" max="18" width="20.703125" customWidth="true" bestFit="true"/>
     <col min="19" max="19" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="20" max="20" width="8.53515625" customWidth="true" bestFit="true"/>
-    <col min="21" max="21" width="14.72265625" customWidth="true" bestFit="true"/>
-    <col min="22" max="22" width="15.13671875" customWidth="true" bestFit="true"/>
-    <col min="23" max="23" width="16.3203125" customWidth="true" bestFit="true"/>
-    <col min="24" max="24" width="16.16796875" customWidth="true" bestFit="true"/>
-    <col min="25" max="25" width="144.1953125" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="42.01953125" customWidth="true" bestFit="true"/>
-    <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
-    <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
-    <col min="29" max="29" width="28.21875" customWidth="true" bestFit="true"/>
-    <col min="30" max="30" width="14.7578125" customWidth="true" bestFit="true"/>
-    <col min="31" max="31" width="12.359375" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="32" max="32" width="29.98828125" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="33" max="33" width="9.046875" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="34" max="34" width="9.46484375" customWidth="true" bestFit="true"/>
+    <col min="20" max="20" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="21" max="21" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="22" max="22" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="23" max="23" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="24" max="24" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="25" max="25" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="27" max="27" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="28" max="28" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="29" max="29" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="30" max="30" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="31" max="31" width="5.0" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="32" max="32" width="5.0" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="33" max="33" width="5.0" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="34" max="34" width="5.0" customWidth="true" bestFit="true"/>
     <col min="35" max="35" width="100.703125" customWidth="true"/>
-    <col min="37" max="37" width="24.1328125" customWidth="true" bestFit="true"/>
-    <col min="38" max="38" width="57.64453125" customWidth="true" bestFit="true"/>
-    <col min="39" max="39" width="36.84375" customWidth="true" bestFit="true"/>
-    <col min="40" max="40" width="31.65234375" customWidth="true" bestFit="true"/>
+    <col min="37" max="37" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="38" max="38" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="39" max="39" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="40" max="40" width="5.0" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
chore: publish ekg IG 2.0.1 (#94)
Co-authored-by: olw-medcom <olw-medcom@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ig/ekg/StructureDefinition-medcom-ekg-recording-bundle.xlsx
+++ b/ig/ekg/StructureDefinition-medcom-ekg-recording-bundle.xlsx
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>2.0.0</t>
+    <t>2.0.1</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-04T11:20:25+00:00</t>
+    <t>2026-10-01T09:27:07+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1315,45 +1315,45 @@
   <dimension ref="A1:AN81"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="62.49609375" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="33.44140625" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="29.421875" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="4" max="4" width="18.19140625" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="5" max="5" width="5.80859375" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="4.23828125" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="4.65625" customWidth="true" bestFit="true"/>
-    <col min="8" max="8" width="13.953125" customWidth="true" bestFit="true"/>
-    <col min="9" max="9" width="11.3671875" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="5.0" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="4" max="4" width="5.0" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="5" max="5" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="9" max="9" width="5.0" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="79.828125" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="5.0" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>
-    <col min="15" max="15" width="255.0" customWidth="true" bestFit="true"/>
+    <col min="15" max="15" width="5.0" customWidth="true" bestFit="true"/>
     <col min="16" max="16" width="20.703125" customWidth="true" bestFit="true"/>
     <col min="17" max="17" width="20.703125" customWidth="true" bestFit="true"/>
     <col min="18" max="18" width="20.703125" customWidth="true" bestFit="true"/>
     <col min="19" max="19" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="20" max="20" width="8.53515625" customWidth="true" bestFit="true"/>
-    <col min="21" max="21" width="14.72265625" customWidth="true" bestFit="true"/>
-    <col min="22" max="22" width="15.13671875" customWidth="true" bestFit="true"/>
-    <col min="23" max="23" width="16.3203125" customWidth="true" bestFit="true"/>
-    <col min="24" max="24" width="16.16796875" customWidth="true" bestFit="true"/>
-    <col min="25" max="25" width="144.1953125" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="42.01953125" customWidth="true" bestFit="true"/>
-    <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
-    <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
-    <col min="29" max="29" width="28.21875" customWidth="true" bestFit="true"/>
-    <col min="30" max="30" width="14.7578125" customWidth="true" bestFit="true"/>
-    <col min="31" max="31" width="12.359375" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="32" max="32" width="29.98828125" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="33" max="33" width="9.046875" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="34" max="34" width="9.46484375" customWidth="true" bestFit="true"/>
+    <col min="20" max="20" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="21" max="21" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="22" max="22" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="23" max="23" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="24" max="24" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="25" max="25" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="27" max="27" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="28" max="28" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="29" max="29" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="30" max="30" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="31" max="31" width="5.0" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="32" max="32" width="5.0" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="33" max="33" width="5.0" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="34" max="34" width="5.0" customWidth="true" bestFit="true"/>
     <col min="35" max="35" width="100.703125" customWidth="true"/>
-    <col min="37" max="37" width="24.1328125" customWidth="true" bestFit="true"/>
-    <col min="38" max="38" width="57.64453125" customWidth="true" bestFit="true"/>
-    <col min="39" max="39" width="36.84375" customWidth="true" bestFit="true"/>
-    <col min="40" max="40" width="31.65234375" customWidth="true" bestFit="true"/>
+    <col min="37" max="37" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="38" max="38" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="39" max="39" width="5.0" customWidth="true" bestFit="true"/>
+    <col min="40" max="40" width="5.0" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>